<commit_message>
Stage 8 review fixes: C-017
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/TP04/MV-2016-095/MV-2016-095_AssayWorksheet_061616_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/TP04/MV-2016-095/MV-2016-095_AssayWorksheet_061616_v03.xlsx
@@ -166,7 +166,7 @@
   <commentList>
     <comment ref="D4" authorId="0" shapeId="0">
       <text>
-        <t>CYP2C19 is the most flagged isoform in this set; flagged compounds carried into the IC50 work.</t>
+        <t>CYP2C19 and CYP3A4 share the highest count above 50% inhibition at 10 µM. CYP3A4 concentration-response results cover the full test article set.</t>
       </text>
     </comment>
   </commentList>
@@ -1585,7 +1585,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reference inhibitors and historical ranges</t>
+          <t>Reference inhibitors and historical comparators</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Most flagged isoform</t>
+          <t>Most flagged isoforms</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">

</xml_diff>